<commit_message>
chore: publish IP review artifacts and history bundles
</commit_message>
<xml_diff>
--- a/src_qor/test-results/formal_nl_20261024/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/latest.xlsx
+++ b/src_qor/test-results/formal_nl_20261024/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/latest.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="262">
   <si>
     <t>00-概览</t>
   </si>
   <si>
-    <t>IP：SRAM22.sram22_1024x32m8w8；Review：review_20261024T123609Z_91f3fe4c；仅汇总本 IP、本次选择的检查。未选择不代表通过。</t>
+    <t>IP：SRAM22.sram22_1024x32m8w8；Review：review_20261024T164723Z_d91a0632；仅汇总本 IP、本次选择的检查。未选择不代表通过。</t>
   </si>
   <si>
     <t>IP</t>
@@ -53,6 +53,9 @@
     <t>执行失败项</t>
   </si>
   <si>
+    <t>质量判断</t>
+  </si>
+  <si>
     <t>正式可见文件</t>
   </si>
   <si>
@@ -62,6 +65,9 @@
     <t>报告结论</t>
   </si>
   <si>
+    <t>sram22_1024x32m8w8</t>
+  </si>
+  <si>
     <t>SRAM22.sram22_1024x32m8w8</t>
   </si>
   <si>
@@ -74,7 +80,10 @@
     <t>lef_review、formal_nl、macro_index、lef_liberty_check</t>
   </si>
   <si>
-    <t>检查任务结果汇总；不等于正式放行或完整性通过</t>
+    <t>发现已确认变化</t>
+  </si>
+  <si>
+    <t>仅评价本次已选检查与输入范围；本次未运行：无。不等同于 IP 全面质量通过或正式发布放行。</t>
   </si>
   <si>
     <t>01-工程检查</t>
@@ -107,7 +116,7 @@
     <t>formal_nl：执行完成；macro_index：执行完成</t>
   </si>
   <si>
-    <t>formal_nl：可见文件 7 个；断链 0 个；macro_index：Macro 1 个；未关联文件 0 个；未映射对象 0 个</t>
+    <t>formal_nl：可见文件 7 个；断链 0 个；macro_index：Macro 1 个；未关联文件 0 个；待核实对象 0 个</t>
   </si>
   <si>
     <t>单次目录或选定版本盘点，不代表完整历史。</t>
@@ -143,7 +152,7 @@
     <t>macro_index：执行完成</t>
   </si>
   <si>
-    <t>macro_index：Macro 1 个；未关联文件 0 个；未映射对象 0 个</t>
+    <t>macro_index：Macro 1 个；未关联文件 0 个；待核实对象 0 个</t>
   </si>
   <si>
     <t>选定 FileMap 的对象与文件关联，不代表多版本演进已覆盖。</t>
@@ -185,7 +194,7 @@
     <t>macro_index：执行完成；lef_liberty_check：执行完成</t>
   </si>
   <si>
-    <t>macro_index：Macro 1 个；未关联文件 0 个；未映射对象 0 个；lef_liberty_check：Liberty 3 个；接口不一致文件 0 个；证据不足文件 0 个；单文件范围差异 0 个</t>
+    <t>macro_index：Macro 1 个；未关联文件 0 个；待核实对象 0 个；lef_liberty_check：Liberty 3 个；接口不一致文件 0 个；证据不足文件 0 个；单文件范围差异 0 个</t>
   </si>
   <si>
     <t>限已选择输入和当前解析字段；不推断未绑定视图。</t>
@@ -251,13 +260,13 @@
     <t>仅比较指定的旧/新 LEF 文件及当前解析器覆盖字段。</t>
   </si>
   <si>
-    <t>{"check": "lef_review", "sources": [{"role": "lef_old", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20241117_cb95ccae/LEF/sram22_1024x32m8w8.lef", "sha256": "b88059d119a6e937507ec8383052c33d88c5a9d3a3a04a1dca6747bb8f5dd4db"}, {"role": "lef_new", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LEF/sram22_1024x32m8w8.lef", "sha256": "bfb5ca9250f9a74d9e9dd134a3c1033cc6fd28299addba55481d10f33591e9bf"}], "source_versions": [], "formal_stages": []}</t>
-  </si>
-  <si>
-    <t>{"old_file": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20241117_cb95ccae/LEF/sram22_1024x32m8w8.lef", "new_file": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LEF/sram22_1024x32m8w8.lef"}</t>
-  </si>
-  <si>
-    <t>/tmp/ai_lib_formal_script_check_es3ct8fp/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/runs/review_20261024T123609Z_91f3fe4c/evidence/lef_review/lef_analysis.json</t>
+    <t>lef_old 1；lef_new 1</t>
+  </si>
+  <si>
+    <t>old_file: sram22_1024x32m8w8.lef；new_file: sram22_1024x32m8w8.lef</t>
+  </si>
+  <si>
+    <t>evidence/lef_review.json</t>
   </si>
   <si>
     <t>formal_nl</t>
@@ -269,31 +278,31 @@
     <t>只读盘点链接和路径；不读取文件内容，也不判断交付齐套或发布放行。</t>
   </si>
   <si>
-    <t>{"check": "formal_nl", "sources": [{"role": "formal_nl_config", "path": "/tmp/ai_lib_formal_script_check_es3ct8fp/sram22_1024x32m8w8_formal.yml"}, {"role": "formal_nl_root", "path": "/home/polaris/proj/mx/ai_lib/lib_NL2.5_3/IP"}, {"role": "formal_raw_source", "version": "20260924_de0a9a7"}, {"role": "formal_stage", "stage": "lib_NL2.5_3"}], "source_versions": ["20260924_de0a9a7"], "formal_stages": ["lib_NL2.5_3"]}</t>
-  </si>
-  <si>
-    <t>{"config": "/tmp/ai_lib_formal_script_check_es3ct8fp/sram22_1024x32m8w8_formal.yml"}</t>
-  </si>
-  <si>
-    <t>/tmp/ai_lib_formal_script_check_es3ct8fp/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/runs/review_20261024T123609Z_91f3fe4c/evidence/formal_nl/formal_nl.json</t>
+    <t>formal_nl_config 1；formal_nl_root 1；formal_raw_source 1；formal_stage 1；版本 20260924_de0a9a7</t>
+  </si>
+  <si>
+    <t>config: SRAM22.sram22_1024x32m8w8__2b292f02b336.yml</t>
+  </si>
+  <si>
+    <t>evidence/formal_nl.json</t>
   </si>
   <si>
     <t>macro_index</t>
   </si>
   <si>
-    <t>Macro 1 个；未关联文件 0 个；未映射对象 0 个</t>
+    <t>Macro 1 个；未关联文件 0 个；待核实对象 0 个</t>
   </si>
   <si>
     <t>按当前解析事实建立名称关联；未映射不等于交付缺失，索引完成不代表全部视图齐套。</t>
   </si>
   <si>
-    <t>{"check": "macro_index", "sources": [{"role": "filemap", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7", "version": "20260924_de0a9a7"}, {"role": "filemap_context", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7"}, {"role": "macro_source", "version": "20260924_de0a9a7"}], "source_versions": ["20260924_de0a9a7"], "formal_stages": []}</t>
-  </si>
-  <si>
-    <t>{"root": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7", "version": "20260924_de0a9a7", "library_id": "SRAM22.sram22_1024x32m8w8"}</t>
-  </si>
-  <si>
-    <t>/tmp/ai_lib_formal_script_check_es3ct8fp/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/runs/review_20261024T123609Z_91f3fe4c/evidence/macro_index.json</t>
+    <t>filemap 1；filemap_context 1；macro_source 1；版本 20260924_de0a9a7</t>
+  </si>
+  <si>
+    <t>root: 20260924_de0a9a7；version: 20260924_de0a9a7；library_id: SRAM22.sram22_1024x32m8w8</t>
+  </si>
+  <si>
+    <t>evidence/macro_index.json</t>
   </si>
   <si>
     <t>lef_liberty_check</t>
@@ -305,13 +314,13 @@
     <t>逐文件核对且不合并 Corner；范围差异不等于缺交付，不判断时序性能或发布放行。</t>
   </si>
   <si>
-    <t>{"check": "lef_liberty_check", "sources": [{"role": "bound_lef", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LEF/sram22_1024x32m8w8.lef", "sha256": "bfb5ca9250f9a74d9e9dd134a3c1033cc6fd28299addba55481d10f33591e9bf"}, {"role": "liberty", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_ff_n40C_1v95.lib"}, {"role": "liberty", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_ss_100C_1v60.lib"}, {"role": "liberty", "path": "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_tt_025C_1v80.lib"}], "source_versions": [], "formal_stages": []}</t>
-  </si>
-  <si>
-    <t>{"liberty_files": ["/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_ff_n40C_1v95.lib", "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_ss_100C_1v60.lib", "/home/polaris/proj/mx/ai_lib/3rd_IP/SRAM22/sram22_1024x32m8w8/20260924_de0a9a7/LIB/NLDM/sram22_1024x32m8w8_tt_025C_1v80.lib"], "include_matching_cells": false}</t>
-  </si>
-  <si>
-    <t>/tmp/ai_lib_formal_script_check_es3ct8fp/libraries/SRAM22.sram22_1024x32m8w8__2b292f02b336/runs/review_20261024T123609Z_91f3fe4c/evidence/lef_liberty_check/lef_liberty_check.json</t>
+    <t>bound_lef 1；liberty 3</t>
+  </si>
+  <si>
+    <t>liberty_files 3 项</t>
+  </si>
+  <si>
+    <t>evidence/lef_liberty_check.json</t>
   </si>
   <si>
     <t>03-问答</t>
@@ -329,6 +338,15 @@
     <t>来源报告</t>
   </si>
   <si>
+    <t>本次有哪些检查没有运行？</t>
+  </si>
+  <si>
+    <t>无，四项检查均已选择执行。</t>
+  </si>
+  <si>
+    <t>未选择或未配置的检查不代表通过或失败；如需结论，先补齐输入并单独执行。</t>
+  </si>
+  <si>
     <t>正式目录观察到哪些文件类型和数量？</t>
   </si>
   <si>
@@ -338,6 +356,15 @@
     <t>阶段 lib_NL2.5_3；目录盘点状态 COMPLETE。数量为可见路径，不判断是否必需。</t>
   </si>
   <si>
+    <t>当前正式文件分别来自哪些 RAW 版本？</t>
+  </si>
+  <si>
+    <t>20260924_de0a9a7：7 个文件</t>
+  </si>
+  <si>
+    <t>仅统计所选正式阶段可见且来源可追溯的文件；不推断内容新旧。</t>
+  </si>
+  <si>
     <t>解析并建立了多少个 LEF Macro 索引？</t>
   </si>
   <si>
@@ -347,6 +374,15 @@
     <t>索引覆盖见 Macro-View 表；文件名/名称关联不代表文件内容确认或交付齐套。</t>
   </si>
   <si>
+    <t>哪些 View 尚未关联到 LEF Macro？</t>
+  </si>
+  <si>
+    <t>CDL：1 个 Macro 未关联；DB：1 个 Macro 未关联</t>
+  </si>
+  <si>
+    <t>未关联只是当前索引范围的名称/解析关联状态，不等于必需文件缺失。</t>
+  </si>
+  <si>
     <t>两份指定 LEF 有哪些已确认变化？</t>
   </si>
   <si>
@@ -356,6 +392,15 @@
     <t>仅限所选的旧/新 LEF 文件及当前 Parser 覆盖字段。</t>
   </si>
   <si>
+    <t>目标 LEF 比基准改了哪些 Macro？</t>
+  </si>
+  <si>
+    <t>新增：无；移除：无；字段变化对象：sram22_1024x32m8w8</t>
+  </si>
+  <si>
+    <t>仅限两份指定 LEF；字段变化不自动代表功能影响。</t>
+  </si>
+  <si>
     <t>指定 Liberty 与 LEF 的接口核对结果是什么？</t>
   </si>
   <si>
@@ -365,6 +410,15 @@
     <t>单文件名称范围差异不等于缺交付；接口结论仅限输入 Liberty 与指定 LEF 的同名对象、当前解析器支持字段；不判断时序性能或放行。</t>
   </si>
   <si>
+    <t>本次 Liberty 识别到哪些工艺角线索？</t>
+  </si>
+  <si>
+    <t>FF, SS, TT；未识别工艺角文件 0 个。</t>
+  </si>
+  <si>
+    <t>角标由文件名/Library 名提取，不代表已确认 Signoff 条件。</t>
+  </si>
+  <si>
     <t>04-关注项</t>
   </si>
   <si>
@@ -396,9 +450,6 @@
   </si>
   <si>
     <t>已确认变化</t>
-  </si>
-  <si>
-    <t>sram22_1024x32m8w8</t>
   </si>
   <si>
     <t>pins.vdd.rects: [{'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 227.6, 'x2': 10.32, 'y2': 227.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 224.88, 'x2': 11.0, 'y2': 225.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 223.52, 'x2': 11.68, 'y2': 223.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 220.8, 'x2': 12.36, 'y2': 221.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 219.44, 'x2': 13.04, 'y2': 219.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 216.72, 'x2': 13.72, 'y2': 217.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 215.36, 'x2': 14.4, 'y2': 215.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 214.0, 'x2': 15.08, 'y2': 214.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 212.64, 'x2': 15.76, 'y2': 212.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 209.92, 'x2': 16.44, 'y2': 210.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 184.08, 'x2': 168.76, 'y2': 184.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 208.56, 'x2': 17.12, 'y2': 208.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 207.2, 'x2': 17.8, 'y2': 207.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 204.48, 'x2': 18.48, 'y2': 204.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 175.92, 'x2': 181.68, 'y2': 176.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 177.28, 'x2': 181.68, 'y2': 177.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 178.64, 'x2': 181.68, 'y2': 178.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 180.0, 'x2': 181.68, 'y2': 180.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 181.36, 'x2': 181.68, 'y2': 181.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 182.72, 'x2': 181.68, 'y2': 183.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 132.4, 'x2': 202.76, 'y2': 132.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 133.76, 'x2': 202.76, 'y2': 134.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 135.12, 'x2': 202.76, 'y2': 135.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 136.48, 'x2': 202.76, 'y2': 136.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 137.84, 'x2': 202.76, 'y2': 138.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 139.2, 'x2': 202.76, 'y2': 139.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 140.56, 'x2': 202.76, 'y2': 140.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 141.92, 'x2': 202.76, 'y2': 142.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 143.28, 'x2': 202.76, 'y2': 143.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 144.64, 'x2': 202.76, 'y2': 144.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 146.0, 'x2': 202.76, 'y2': 146.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 147.36, 'x2': 202.76, 'y2': 147.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 148.72, 'x2': 202.76, 'y2': 149.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 150.08, 'x2': 202.76, 'y2': 150.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 151.44, 'x2': 202.76, 'y2': 151.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 152.8, 'x2': 202.76, 'y2': 153.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 154.16, 'x2': 202.76, 'y2': 154.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 155.52, 'x2': 202.76, 'y2': 155.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 156.88, 'x2': 202.76, 'y2': 157.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 158.24, 'x2': 202.76, 'y2': 158.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 159.6, 'x2': 202.76, 'y2': 159.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 160.96, 'x2': 202.76, 'y2': 161.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 162.32, 'x2': 202.76, 'y2': 162.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 163.68, 'x2': 202.76, 'y2': 164.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 165.04, 'x2': 202.76, 'y2': 165.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 166.4, 'x2': 202.76, 'y2': 166.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 167.76, 'x2': 202.76, 'y2': 168.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 169.12, 'x2': 202.76, 'y2': 169.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 170.48, 'x2': 202.76, 'y2': 170.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 171.84, 'x2': 202.76, 'y2': 172.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 185.44, 'x2': 215.0, 'y2': 185.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 97.04, 'x2': 223.16, 'y2': 97.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 107.92, 'x2': 223.84, 'y2': 108.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 112.0, 'x2': 223.84, 'y2': 112.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 129.68, 'x2': 223.84, 'y2': 130.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 86.16, 'x2': 223.84, 'y2': 86.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 124.24, 'x2': 225.2, 'y2': 124.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 87.52, 'x2': 225.2, 'y2': 87.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 118.8, 'x2': 225.88, 'y2': 119.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 46.72, 'x2': 225.88, 'y2': 47.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 94.32, 'x2': 225.88, 'y2': 94.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 117.44, 'x2': 226.56, 'y2': 117.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 128.32, 'x2': 227.24, 'y2': 128.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 173.2, 'x2': 227.24, 'y2': 173.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 48.08, 'x2': 227.24, 'y2': 48.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 88.88, 'x2': 227.24, 'y2': 89.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 120.16, 'x2': 228.6, 'y2': 120.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 92.96, 'x2': 228.6, 'y2': 93.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 103.84, 'x2': 229.96, 'y2': 104.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 114.72, 'x2': 230.64, 'y2': 115.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 105.2, 'x2': 232.68, 'y2': 105.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 109.28, 'x2': 232.68, 'y2': 109.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 113.36, 'x2': 232.68, 'y2': 113.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 122.88, 'x2': 232.68, 'y2': 123.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 126.96, 'x2': 232.68, 'y2': 127.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 99.76, 'x2': 232.68, 'y2': 100.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 102.48, 'x2': 233.36, 'y2': 102.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 91.6, 'x2': 233.36, 'y2': 91.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 98.4, 'x2': 233.36, 'y2': 98.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 106.56, 'x2': 236.08, 'y2': 106.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 110.64, 'x2': 244.92, 'y2': 110.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 54.88, 'x2': 246.96, 'y2': 55.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 61.68, 'x2': 248.32, 'y2': 62.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 45.36, 'x2': 249.0, 'y2': 45.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 63.04, 'x2': 249.68, 'y2': 63.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 192.24, 'x2': 25.28, 'y2': 192.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 193.6, 'x2': 25.28, 'y2': 193.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 194.96, 'x2': 25.28, 'y2': 195.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 196.32, 'x2': 25.28, 'y2': 196.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 197.68, 'x2': 25.28, 'y2': 198.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 199.04, 'x2': 25.28, 'y2': 199.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 200.4, 'x2': 25.28, 'y2': 200.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 44.0, 'x2': 250.36, 'y2': 44.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 64.4, 'x2': 251.04, 'y2': 64.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 42.64, 'x2': 251.72, 'y2': 42.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 101.12, 'x2': 263.28, 'y2': 101.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 65.76, 'x2': 263.28, 'y2': 66.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 67.12, 'x2': 263.28, 'y2': 67.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 68.48, 'x2': 263.28, 'y2': 68.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 69.84, 'x2': 263.28, 'y2': 70.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 71.2, 'x2': 263.28, 'y2': 71.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 72.56, 'x2': 263.28, 'y2': 72.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 73.92, 'x2': 263.28, 'y2': 74.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 75.28, 'x2': 263.28, 'y2': 75.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 76.64, 'x2': 263.28, 'y2': 76.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 78.0, 'x2': 263.28, 'y2': 78.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 79.36, 'x2': 263.28, 'y2': 79.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 80.72, 'x2': 263.28, 'y2': 81.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 82.08, 'x2': 263.28, 'y2': 82.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 83.44, 'x2': 263.28, 'y2': 83.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 84.8, 'x2': 263.28, 'y2': 85.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 90.24, 'x2': 263.28, 'y2': 90.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 95.68, 'x2': 263.28, 'y2': 96.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 190.88, 'x2': 27.32, 'y2': 191.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 20.88, 'x2': 289.12, 'y2': 21.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 24.96, 'x2': 289.12, 'y2': 25.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 174.56, 'x2': 297.28, 'y2': 174.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 52.16, 'x2': 355.76, 'y2': 52.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 53.52, 'x2': 355.76, 'y2': 53.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 265.68, 'x2': 36.16, 'y2': 266.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 10.0, 'x2': 363.92, 'y2': 10.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 264.32, 'x2': 37.52, 'y2': 264.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 125.6, 'x2': 372.08, 'y2': 125.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 262.96, 'x2': 38.88, 'y2': 263.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 121.52, 'x2': 382.96, 'y2': 121.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 186.8, 'x2': 388.4, 'y2': 187.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 188.16, 'x2': 388.4, 'y2': 188.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 189.52, 'x2': 388.4, 'y2': 189.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 446.56, 'x2': 388.4, 'y2': 446.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 447.92, 'x2': 388.4, 'y2': 448.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 27.68, 'x2': 390.44, 'y2': 28.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 11.36, 'x2': 391.12, 'y2': 11.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 116.08, 'x2': 391.12, 'y2': 116.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 12.72, 'x2': 391.12, 'y2': 13.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 131.04, 'x2': 391.12, 'y2': 131.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 14.08, 'x2': 391.12, 'y2': 14.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 15.44, 'x2': 391.12, 'y2': 15.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 16.8, 'x2': 391.12, 'y2': 17.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 18.16, 'x2': 391.12, 'y2': 18.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 19.52, 'x2': 391.12, 'y2': 19.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 22.24, 'x2': 391.12, 'y2': 22.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 23.6, 'x2': 391.12, 'y2': 23.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 26.32, 'x2': 391.12, 'y2': 26.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 29.04, 'x2': 391.12, 'y2': 29.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 30.4, 'x2': 391.12, 'y2': 30.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 31.76, 'x2': 391.12, 'y2': 32.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 33.12, 'x2': 391.12, 'y2': 33.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 34.48, 'x2': 391.12, 'y2': 34.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 35.84, 'x2': 391.12, 'y2': 36.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 37.2, 'x2': 391.12, 'y2': 37.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 38.56, 'x2': 391.12, 'y2': 38.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 39.92, 'x2': 391.12, 'y2': 40.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 41.28, 'x2': 391.12, 'y2': 41.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 49.44, 'x2': 391.12, 'y2': 49.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 50.8, 'x2': 391.12, 'y2': 51.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 56.24, 'x2': 391.12, 'y2': 56.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 57.6, 'x2': 391.12, 'y2': 57.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 58.96, 'x2': 391.12, 'y2': 59.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 60.32, 'x2': 391.12, 'y2': 60.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 5.92, 'x2': 404.04, 'y2': 6.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 211.28, 'x2': 59.28, 'y2': 211.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 201.76, 'x2': 75.6, 'y2': 202.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 203.12, 'x2': 75.6, 'y2': 203.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 205.84, 'x2': 75.6, 'y2': 206.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 218.08, 'x2': 75.6, 'y2': 218.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 222.16, 'x2': 75.6, 'y2': 222.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 226.24, 'x2': 75.6, 'y2': 226.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 230.32, 'x2': 75.6, 'y2': 230.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 231.68, 'x2': 75.6, 'y2': 232.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 233.04, 'x2': 75.6, 'y2': 233.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 234.4, 'x2': 75.6, 'y2': 234.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 235.76, 'x2': 75.6, 'y2': 236.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 237.12, 'x2': 75.6, 'y2': 237.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 238.48, 'x2': 75.6, 'y2': 238.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 239.84, 'x2': 75.6, 'y2': 240.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 241.2, 'x2': 75.6, 'y2': 241.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 242.56, 'x2': 75.6, 'y2': 242.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 243.92, 'x2': 75.6, 'y2': 244.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 245.28, 'x2': 75.6, 'y2': 245.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 248.0, 'x2': 75.6, 'y2': 248.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 249.36, 'x2': 75.6, 'y2': 249.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 250.72, 'x2': 75.6, 'y2': 251.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 252.08, 'x2': 75.6, 'y2': 252.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 253.44, 'x2': 75.6, 'y2': 253.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 268.4, 'x2': 75.6, 'y2': 268.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 269.76, 'x2': 75.6, 'y2': 270.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 272.48, 'x2': 75.6, 'y2': 272.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 273.84, 'x2': 75.6, 'y2': 274.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 275.2, 'x2': 75.6, 'y2': 275.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 276.56, 'x2': 75.6, 'y2': 276.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 277.92, 'x2': 75.6, 'y2': 278.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 280.64, 'x2': 75.6, 'y2': 280.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 282.0, 'x2': 75.6, 'y2': 282.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 283.36, 'x2': 75.6, 'y2': 283.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 284.72, 'x2': 75.6, 'y2': 285.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 288.8, 'x2': 75.6, 'y2': 289.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 290.16, 'x2': 75.6, 'y2': 290.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 291.52, 'x2': 75.6, 'y2': 291.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 292.88, 'x2': 75.6, 'y2': 293.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 296.96, 'x2': 75.6, 'y2': 297.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 298.32, 'x2': 75.6, 'y2': 298.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 299.68, 'x2': 75.6, 'y2': 300.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 301.04, 'x2': 75.6, 'y2': 301.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 303.76, 'x2': 75.6, 'y2': 304.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 305.12, 'x2': 75.6, 'y2': 305.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 307.84, 'x2': 75.6, 'y2': 308.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 309.2, 'x2': 75.6, 'y2': 309.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 311.92, 'x2': 75.6, 'y2': 312.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 313.28, 'x2': 75.6, 'y2': 313.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 314.64, 'x2': 75.6, 'y2': 314.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 316.0, 'x2': 75.6, 'y2': 316.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 317.36, 'x2': 75.6, 'y2': 317.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 320.08, 'x2': 75.6, 'y2': 320.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 321.44, 'x2': 75.6, 'y2': 321.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 322.8, 'x2': 75.6, 'y2': 323.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 324.16, 'x2': 75.6, 'y2': 324.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 0.16, 'x2': 764.08, 'y2': 1.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 449.28, 'x2': 764.08, 'y2': 449.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 450.64, 'x2': 764.08, 'y2': 450.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 452.0, 'x2': 764.08, 'y2': 452.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 453.36, 'x2': 764.08, 'y2': 453.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 454.72, 'x2': 764.08, 'y2': 455.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 458.76, 'x2': 764.08, 'y2': 460.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 7.28, 'x2': 764.08, 'y2': 7.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 8.64, 'x2': 764.08, 'y2': 8.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 256.16, 'x2': 77.64, 'y2': 256.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 257.52, 'x2': 77.64, 'y2': 257.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 258.88, 'x2': 77.64, 'y2': 259.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 261.6, 'x2': 77.64, 'y2': 261.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 267.04, 'x2': 77.64, 'y2': 267.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 287.44, 'x2': 77.64, 'y2': 287.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 295.6, 'x2': 77.64, 'y2': 295.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 306.48, 'x2': 77.64, 'y2': 306.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 326.88, 'x2': 78.32, 'y2': 327.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 330.96, 'x2': 78.32, 'y2': 331.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 332.32, 'x2': 78.32, 'y2': 332.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 335.04, 'x2': 78.32, 'y2': 335.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 336.4, 'x2': 78.32, 'y2': 336.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 337.76, 'x2': 78.32, 'y2': 338.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 340.48, 'x2': 78.32, 'y2': 340.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 343.2, 'x2': 78.32, 'y2': 343.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 344.56, 'x2': 78.32, 'y2': 344.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 345.92, 'x2': 78.32, 'y2': 346.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 347.28, 'x2': 78.32, 'y2': 347.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 351.36, 'x2': 79.0, 'y2': 351.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 352.72, 'x2': 79.0, 'y2': 353.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 354.08, 'x2': 79.0, 'y2': 354.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 355.44, 'x2': 79.0, 'y2': 355.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 359.52, 'x2': 79.0, 'y2': 359.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 360.88, 'x2': 79.0, 'y2': 361.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 362.24, 'x2': 79.0, 'y2': 362.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 363.6, 'x2': 79.0, 'y2': 363.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 366.32, 'x2': 79.0, 'y2': 366.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 369.04, 'x2': 79.0, 'y2': 369.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 370.4, 'x2': 79.0, 'y2': 370.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 371.76, 'x2': 79.0, 'y2': 372.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 374.48, 'x2': 79.0, 'y2': 374.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 375.84, 'x2': 79.0, 'y2': 376.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 379.92, 'x2': 79.0, 'y2': 380.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 382.64, 'x2': 79.0, 'y2': 382.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 384.0, 'x2': 79.0, 'y2': 384.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 385.36, 'x2': 79.0, 'y2': 385.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 390.8, 'x2': 79.0, 'y2': 391.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 392.16, 'x2': 79.0, 'y2': 392.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 393.52, 'x2': 79.0, 'y2': 393.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 394.88, 'x2': 79.0, 'y2': 395.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 398.96, 'x2': 79.0, 'y2': 399.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 400.32, 'x2': 79.0, 'y2': 400.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 401.68, 'x2': 79.0, 'y2': 402.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 403.04, 'x2': 79.0, 'y2': 403.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 405.76, 'x2': 79.0, 'y2': 406.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 408.48, 'x2': 79.0, 'y2': 408.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 409.84, 'x2': 79.0, 'y2': 410.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 411.2, 'x2': 79.0, 'y2': 411.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 413.92, 'x2': 79.68, 'y2': 414.24}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 415.28, 'x2': 79.68, 'y2': 415.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 418.0, 'x2': 79.68, 'y2': 418.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 419.36, 'x2': 79.68, 'y2': 419.68}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 422.08, 'x2': 79.68, 'y2': 422.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 423.44, 'x2': 79.68, 'y2': 423.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 424.8, 'x2': 79.68, 'y2': 425.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 427.52, 'x2': 79.68, 'y2': 427.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 430.24, 'x2': 79.68, 'y2': 430.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 431.6, 'x2': 79.68, 'y2': 431.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 432.96, 'x2': 79.68, 'y2': 433.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 434.32, 'x2': 79.68, 'y2': 434.64}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 438.4, 'x2': 79.68, 'y2': 438.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 439.76, 'x2': 79.68, 'y2': 440.08}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 441.12, 'x2': 79.68, 'y2': 441.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 442.48, 'x2': 79.68, 'y2': 442.8}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 318.72, 'x2': 80.36, 'y2': 319.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 350.0, 'x2': 80.36, 'y2': 350.32}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 416.64, 'x2': 81.04, 'y2': 416.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 260.24, 'x2': 81.72, 'y2': 260.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 386.72, 'x2': 81.72, 'y2': 387.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 328.24, 'x2': 82.4, 'y2': 328.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 358.16, 'x2': 82.4, 'y2': 358.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 389.44, 'x2': 82.4, 'y2': 389.76}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 329.6, 'x2': 83.08, 'y2': 329.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 271.12, 'x2': 83.76, 'y2': 271.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 397.6, 'x2': 83.76, 'y2': 397.92}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 426.16, 'x2': 83.76, 'y2': 426.48}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 367.68, 'x2': 84.44, 'y2': 368.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 279.28, 'x2': 85.8, 'y2': 279.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 310.56, 'x2': 85.8, 'y2': 310.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 339.12, 'x2': 85.8, 'y2': 339.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 437.04, 'x2': 85.8, 'y2': 437.36}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 407.12, 'x2': 86.48, 'y2': 407.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 377.2, 'x2': 87.16, 'y2': 377.52}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 378.56, 'x2': 87.16, 'y2': 378.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 228.96, 'x2': 9.64, 'y2': 229.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 246.64, 'x2': 99.4, 'y2': 246.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 254.8, 'x2': 99.4, 'y2': 255.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 286.08, 'x2': 99.4, 'y2': 286.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 294.24, 'x2': 99.4, 'y2': 294.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 302.4, 'x2': 99.4, 'y2': 302.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 325.52, 'x2': 99.4, 'y2': 325.84}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 333.68, 'x2': 99.4, 'y2': 334.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 341.84, 'x2': 99.4, 'y2': 342.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 348.64, 'x2': 99.4, 'y2': 348.96}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 356.8, 'x2': 99.4, 'y2': 357.12}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 364.96, 'x2': 99.4, 'y2': 365.28}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 373.12, 'x2': 99.4, 'y2': 373.44}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 381.28, 'x2': 99.4, 'y2': 381.6}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 388.08, 'x2': 99.4, 'y2': 388.4}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 396.24, 'x2': 99.4, 'y2': 396.56}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 404.4, 'x2': 99.4, 'y2': 404.72}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 412.56, 'x2': 99.4, 'y2': 412.88}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 420.72, 'x2': 99.4, 'y2': 421.04}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 428.88, 'x2': 99.4, 'y2': 429.2}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 435.68, 'x2': 99.4, 'y2': 436.0}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 443.84, 'x2': 99.4, 'y2': 444.16}, {'port_index': 0, 'layer': 'met2', 'x1': 0.16, 'y1': 445.2, 'x2': 99.4, 'y2': 445.52}, {'port_index': 0, 'layer': 'met2', 'x1': 103.59, 'y1': 190.595, 'x2': 105.51, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 113.805, 'y1': 190.595, 'x2': 115.725, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 117.645, 'y1': 190.595, 'x2': 119.565, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 130.055, 'y1': 190.595, 'x2': 131.975, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 133.895, 'y1': 190.595, 'x2': 135.815, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 137.735, 'y1': 190.595, 'x2': 139.655, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 141.575, 'y1': 190.595, 'x2': 143.495, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 159.22, 'y1': 190.595, 'x2': 161.14, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 163.06, 'y1': 190.595, 'x2': 164.98, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 166.9, 'y1': 190.595, 'x2': 168.82, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 170.74, 'y1': 190.595, 'x2': 172.66, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 174.58, 'y1': 190.595, 'x2': 176.5, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 178.42, 'y1': 190.595, 'x2': 180.34, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 182.05, 'y1': 180.275, 'x2': 201.69, 'y2': 182.985}, {'port_index': 0, 'layer': 'met2', 'x1': 182.26, 'y1': 190.595, 'x2': 184.18, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 207.2, 'x2': 34.12, 'y2': 207.52}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 208.56, 'x2': 34.12, 'y2': 208.88}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 209.92, 'x2': 34.12, 'y2': 210.24}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 212.64, 'x2': 34.12, 'y2': 212.96}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 214.0, 'x2': 34.12, 'y2': 214.32}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 223.52, 'x2': 34.12, 'y2': 223.84}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 224.88, 'x2': 34.12, 'y2': 225.2}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 227.6, 'x2': 34.12, 'y2': 227.92}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 228.96, 'x2': 34.12, 'y2': 229.28}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 204.48, 'x2': 75.6, 'y2': 204.8}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 216.72, 'x2': 75.6, 'y2': 217.04}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 219.44, 'x2': 75.6, 'y2': 219.76}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 220.8, 'x2': 75.6, 'y2': 221.12}, {'port_index': 0, 'layer': 'met2', 'x1': 20.88, 'y1': 215.36, 'x2': 99.4, 'y2': 215.68}, {'port_index': 0, 'layer': 'met2', 'x1': 202.44, 'y1': 178.64, 'x2': 208.2, 'y2': 178.96}, {'port_index': 0, 'layer': 'met2', 'x1': 202.44, 'y1': 182.72, 'x2': 208.2, 'y2': 183.04}, {'port_index': 0, 'layer': 'met2', 'x1': 202.44, 'y1': 177.28, 'x2': 229.96, 'y2': 177.6}, {'port_index': 0, 'layer': 'met2', 'x1': 202.44, 'y1': 175.92, 'x2': 297.28, 'y2': 176.24}, {'port_index': 0, 'layer': 'met2', 'x1': 203.65, 'y1': 180.575, 'x2': 219.69, 'y2': 181.425}, {'port_index': 0, 'layer': 'met2', 'x1': 209.07, 'y1': 190.595, 'x2': 210.99, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 212.91, 'y1': 190.595, 'x2': 214.83, 'y2': 444.975}, {'port_index': 0, 'layer': 'met2', 'x1': 215.36, 'y1': 184.08,</t>
@@ -667,10 +718,19 @@
     <t>RC角线索</t>
   </si>
   <si>
-    <t>PVT</t>
-  </si>
-  <si>
-    <t>Cell数</t>
+    <t>条件</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Voltage (V)</t>
+  </si>
+  <si>
+    <t>Temp (°C)</t>
+  </si>
+  <si>
+    <t>文件Cell数</t>
   </si>
   <si>
     <t>同名Cell</t>
@@ -706,22 +766,22 @@
     <t>未识别</t>
   </si>
   <si>
-    <t>{"sram22_1024x32m8w8": {"PVT_1P95V_-40C": {"name": "PVT_1P95V_-40C", "process": "1", "temperature": "-40", "voltage": "1.95"}}}</t>
-  </si>
-  <si>
-    <t>工艺角仅为名称线索，不等于人工确认</t>
+    <t>PVT_1P95V_-40C</t>
+  </si>
+  <si>
+    <t>工艺角仅为名称线索；P/V/T 为 Liberty 声明值，不代表签核确认</t>
   </si>
   <si>
     <t>SS</t>
   </si>
   <si>
-    <t>{"sram22_1024x32m8w8": {"PVT_1P6V_100C": {"name": "PVT_1P6V_100C", "process": "1", "temperature": "100", "voltage": "1.6"}}}</t>
+    <t>PVT_1P6V_100C</t>
   </si>
   <si>
     <t>TT</t>
   </si>
   <si>
-    <t>{"sram22_1024x32m8w8": {"PVT_1P8V_25C": {"name": "PVT_1P8V_25C", "process": "1", "temperature": "25", "voltage": "1.8"}}}</t>
+    <t>PVT_1P8V_25C</t>
   </si>
   <si>
     <t>10-Liberty单元</t>
@@ -743,6 +803,15 @@
   </si>
   <si>
     <t>接口状态</t>
+  </si>
+  <si>
+    <t>差异类型</t>
+  </si>
+  <si>
+    <t>具体差异</t>
+  </si>
+  <si>
+    <t>MATCH</t>
   </si>
 </sst>
 </file>
@@ -840,9 +909,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewTable1" displayName="ReviewTable1" ref="A4:J5" totalsRowShown="0">
-  <autoFilter ref="A4:J5"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewTable1" displayName="ReviewTable1" ref="A4:K5" totalsRowShown="0">
+  <autoFilter ref="A4:K5"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="IP"/>
     <tableColumn id="2" name="库标识"/>
     <tableColumn id="3" name="RAW版本"/>
@@ -850,43 +919,47 @@
     <tableColumn id="5" name="已选检查"/>
     <tableColumn id="6" name="执行完成项"/>
     <tableColumn id="7" name="执行失败项"/>
-    <tableColumn id="8" name="正式可见文件"/>
-    <tableColumn id="9" name="Macro数"/>
-    <tableColumn id="10" name="报告结论"/>
+    <tableColumn id="8" name="质量判断"/>
+    <tableColumn id="9" name="正式可见文件"/>
+    <tableColumn id="10" name="Macro数"/>
+    <tableColumn id="11" name="报告结论"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ReviewTable10" displayName="ReviewTable10" ref="A4:P7" totalsRowShown="0">
-  <autoFilter ref="A4:P7"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ReviewTable10" displayName="ReviewTable10" ref="A4:S7" totalsRowShown="0">
+  <autoFilter ref="A4:S7"/>
+  <tableColumns count="19">
     <tableColumn id="1" name="IP"/>
     <tableColumn id="2" name="Liberty文件"/>
     <tableColumn id="3" name="Library"/>
     <tableColumn id="4" name="工艺角线索"/>
     <tableColumn id="5" name="RC角线索"/>
-    <tableColumn id="6" name="PVT"/>
-    <tableColumn id="7" name="Cell数"/>
-    <tableColumn id="8" name="同名Cell"/>
-    <tableColumn id="9" name="LEF有而本文件无"/>
-    <tableColumn id="10" name="本文件有而LEF无"/>
-    <tableColumn id="11" name="信号Pin对照"/>
-    <tableColumn id="12" name="信号Pin差异"/>
-    <tableColumn id="13" name="电源/地脚对照"/>
-    <tableColumn id="14" name="电源/地脚差异"/>
-    <tableColumn id="15" name="证据不足Cell数"/>
-    <tableColumn id="16" name="角标说明"/>
+    <tableColumn id="6" name="条件"/>
+    <tableColumn id="7" name="Process"/>
+    <tableColumn id="8" name="Voltage (V)"/>
+    <tableColumn id="9" name="Temp (°C)"/>
+    <tableColumn id="10" name="文件Cell数"/>
+    <tableColumn id="11" name="同名Cell"/>
+    <tableColumn id="12" name="LEF有而本文件无"/>
+    <tableColumn id="13" name="本文件有而LEF无"/>
+    <tableColumn id="14" name="信号Pin对照"/>
+    <tableColumn id="15" name="信号Pin差异"/>
+    <tableColumn id="16" name="电源/地脚对照"/>
+    <tableColumn id="17" name="电源/地脚差异"/>
+    <tableColumn id="18" name="证据不足Cell数"/>
+    <tableColumn id="19" name="角标说明"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ReviewTable11" displayName="ReviewTable11" ref="A4:I5" totalsRowShown="0">
-  <autoFilter ref="A4:I5"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ReviewTable11" displayName="ReviewTable11" ref="A4:K7" totalsRowShown="0">
+  <autoFilter ref="A4:K7"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="IP"/>
     <tableColumn id="2" name="Liberty文件"/>
     <tableColumn id="3" name="Corner线索"/>
@@ -895,7 +968,9 @@
     <tableColumn id="6" name="信号Pin数"/>
     <tableColumn id="7" name="PG Pin数"/>
     <tableColumn id="8" name="接口状态"/>
-    <tableColumn id="9" name="证据路径"/>
+    <tableColumn id="9" name="差异类型"/>
+    <tableColumn id="10" name="具体差异"/>
+    <tableColumn id="11" name="证据路径"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -935,8 +1010,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ReviewTable4" displayName="ReviewTable4" ref="A4:E8" totalsRowShown="0">
-  <autoFilter ref="A4:E8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ReviewTable4" displayName="ReviewTable4" ref="A4:E13" totalsRowShown="0">
+  <autoFilter ref="A4:E13"/>
   <tableColumns count="5">
     <tableColumn id="1" name="IP"/>
     <tableColumn id="2" name="问题"/>
@@ -1329,18 +1404,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" style="1" customWidth="1"/>
-    <col min="6" max="9" width="12.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="24.7109375" style="1" customWidth="1"/>
+    <col min="6" max="7" width="12.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
+    <col min="9" max="10" width="12.7109375" style="2" customWidth="1"/>
+    <col min="11" max="11" width="47.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27.75" customHeight="1">
+    <row r="1" spans="1:11" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1353,8 +1431,9 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
-    </row>
-    <row r="2" spans="1:10" ht="33.75" customHeight="1">
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1367,8 +1446,9 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
-    </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" ht="32.25" customHeight="1">
+      <c r="K2" s="4"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1399,22 +1479,25 @@
       <c r="J4" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="32.25" customHeight="1">
+      <c r="K4" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="32" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="2">
         <v>4</v>
@@ -1422,20 +1505,23 @@
       <c r="G5" s="2">
         <v>0</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="2">
         <v>7</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <v>1</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>16</v>
+      <c r="K5" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1446,21 +1532,23 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="50.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="50.7109375" style="1" customWidth="1"/>
-    <col min="7" max="15" width="12.7109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="19.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" style="2" customWidth="1"/>
+    <col min="9" max="18" width="12.7109375" style="2" customWidth="1"/>
+    <col min="19" max="19" width="39.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27.75" customHeight="1">
+    <row r="1" spans="1:19" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1477,8 +1565,11 @@
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
-    </row>
-    <row r="2" spans="1:16" ht="33.75" customHeight="1">
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+    </row>
+    <row r="2" spans="1:19" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1497,211 +1588,250 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
-    </row>
-    <row r="4" spans="1:16" s="5" customFormat="1" ht="32.25" customHeight="1">
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+    </row>
+    <row r="4" spans="1:19" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="60" customHeight="1">
+        <v>240</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="60" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>226</v>
+        <v>246</v>
       </c>
       <c r="G5" s="2">
         <v>1</v>
       </c>
       <c r="H5" s="2">
+        <v>1.95</v>
+      </c>
+      <c r="I5" s="2">
+        <v>-40</v>
+      </c>
+      <c r="J5" s="2">
         <v>1</v>
       </c>
-      <c r="I5" s="2">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
       <c r="K5" s="2">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="L5" s="2">
         <v>0</v>
       </c>
       <c r="M5" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N5" s="2">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="O5" s="2">
         <v>0</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="60" customHeight="1">
+      <c r="P5" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="60" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>228</v>
+        <v>248</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
       </c>
       <c r="H6" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="I6" s="2">
+        <v>100</v>
+      </c>
+      <c r="J6" s="2">
         <v>1</v>
       </c>
-      <c r="I6" s="2">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0</v>
-      </c>
       <c r="K6" s="2">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="L6" s="2">
         <v>0</v>
       </c>
       <c r="M6" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N6" s="2">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="O6" s="2">
         <v>0</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="60" customHeight="1">
+      <c r="P6" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="60" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="G7" s="2">
         <v>1</v>
       </c>
       <c r="H7" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="I7" s="2">
+        <v>25</v>
+      </c>
+      <c r="J7" s="2">
         <v>1</v>
       </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0</v>
-      </c>
       <c r="K7" s="2">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2">
         <v>0</v>
       </c>
       <c r="M7" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N7" s="2">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="O7" s="2">
         <v>0</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>227</v>
+      <c r="P7" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:S2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1712,15 +1842,22 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="9" width="12.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="1" customWidth="1"/>
+    <col min="6" max="7" width="12.7109375" style="2" customWidth="1"/>
+    <col min="8" max="10" width="12.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="33.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.75" customHeight="1">
+    <row r="1" spans="1:11" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>232</v>
+        <v>252</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1730,8 +1867,10 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
-    </row>
-    <row r="2" spans="1:9" ht="33.75" customHeight="1">
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1743,40 +1882,135 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-    </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" ht="32.25" customHeight="1">
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>237</v>
+        <v>257</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>121</v>
+        <v>259</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="60" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>82</v>
+      </c>
+      <c r="G5" s="2">
+        <v>2</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>82</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>82</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1798,9 +2032,9 @@
     <col min="6" max="6" width="36.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="27.75" customHeight="1">
+    <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1808,7 +2042,7 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:6" ht="33.75" customHeight="1">
+    <row r="2" spans="1:6" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1818,164 +2052,164 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="4" spans="1:6" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:6" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="45.75" customHeight="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="46" customHeight="1">
       <c r="A5" s="2">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="45.75" customHeight="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="46" customHeight="1">
       <c r="A6" s="2">
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="32.25" customHeight="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="32" customHeight="1">
       <c r="A7" s="2">
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="32.25" customHeight="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="32" customHeight="1">
       <c r="A8" s="2">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="32.25" customHeight="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="32" customHeight="1">
       <c r="A9" s="2">
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="45.75" customHeight="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="46" customHeight="1">
       <c r="A10" s="2">
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="32.25" customHeight="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="32" customHeight="1">
       <c r="A11" s="2">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="60" customHeight="1">
@@ -1983,56 +2217,56 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="32.25" customHeight="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="32" customHeight="1">
       <c r="A13" s="2">
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="32.25" customHeight="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="32" customHeight="1">
       <c r="A14" s="2">
         <v>10</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2052,18 +2286,19 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="43.7109375" style="1" customWidth="1"/>
-    <col min="7" max="9" width="50.7109375" style="1" customWidth="1"/>
+    <col min="7" max="8" width="50.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="33.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.75" customHeight="1">
+    <row r="1" spans="1:9" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2074,7 +2309,7 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" ht="33.75" customHeight="1">
+    <row r="2" spans="1:9" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2087,149 +2322,149 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:9" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="87.75" customHeight="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="46" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="46" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="87.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="87.75" customHeight="1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="87.75" customHeight="1">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="32" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2246,24 +2481,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="5" width="50.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="50.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.75" customHeight="1">
+    <row r="1" spans="1:5" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5" ht="33.75" customHeight="1">
+    <row r="2" spans="1:5" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2272,89 +2508,171 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="4" spans="1:5" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:5" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="32" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="46" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="32" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="32" customHeight="1">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="32" customHeight="1">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="32" customHeight="1">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="32" customHeight="1">
+      <c r="A11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="46" customHeight="1">
+      <c r="A12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="74.25" customHeight="1">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="74.25" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="74.25" customHeight="1">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="74.25" customHeight="1">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>95</v>
+    </row>
+    <row r="13" spans="1:5" ht="32" customHeight="1">
+      <c r="A13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2374,7 +2692,7 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" style="2" customWidth="1"/>
@@ -2383,9 +2701,9 @@
     <col min="9" max="9" width="50.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.75" customHeight="1">
+    <row r="1" spans="1:9" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2396,7 +2714,7 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" ht="33.75" customHeight="1">
+    <row r="2" spans="1:9" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2409,91 +2727,91 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:9" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="87.75" customHeight="1">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="88" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2">
         <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="87.75" customHeight="1">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="88" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2">
         <v>1</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2513,7 +2831,7 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="44.7109375" style="1" customWidth="1"/>
@@ -2523,9 +2841,9 @@
     <col min="11" max="11" width="50.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.75" customHeight="1">
+    <row r="1" spans="1:11" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2538,7 +2856,7 @@
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:11" ht="33.75" customHeight="1">
+    <row r="2" spans="1:11" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2553,7 +2871,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
     </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:11" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -2561,63 +2879,63 @@
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="87.75" customHeight="1">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="88" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -2637,7 +2955,7 @@
   <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="1" customWidth="1"/>
@@ -2648,9 +2966,9 @@
     <col min="10" max="10" width="50.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27.75" customHeight="1">
+    <row r="1" spans="1:10" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2662,7 +2980,7 @@
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:10" ht="33.75" customHeight="1">
+    <row r="2" spans="1:10" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2676,7 +2994,7 @@
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:10" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -2684,220 +3002,220 @@
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="60" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="60" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="60" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="60" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="60" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="60" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2917,7 +3235,7 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="41.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="1" customWidth="1"/>
@@ -2926,9 +3244,9 @@
     <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.75" customHeight="1">
+    <row r="1" spans="1:8" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2938,7 +3256,7 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:8" ht="33.75" customHeight="1">
+    <row r="2" spans="1:8" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2950,7 +3268,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
     </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:8" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -2958,204 +3276,204 @@
         <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="60" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>182</v>
+        <v>199</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="60" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>184</v>
+        <v>201</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="60" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>185</v>
+        <v>202</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>186</v>
+        <v>203</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="60" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>187</v>
+        <v>204</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="60" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -3175,7 +3493,7 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="50.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="1" customWidth="1"/>
@@ -3185,9 +3503,9 @@
     <col min="13" max="13" width="40.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27.75" customHeight="1">
+    <row r="1" spans="1:13" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3202,7 +3520,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
     </row>
-    <row r="2" spans="1:13" ht="33.75" customHeight="1">
+    <row r="2" spans="1:13" ht="34" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -3219,62 +3537,62 @@
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
     </row>
-    <row r="4" spans="1:13" s="5" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:13" s="5" customFormat="1" ht="32" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="60" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="F5" s="2">
         <v>764.24</v>
@@ -3283,7 +3601,7 @@
         <v>460.28</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="I5" s="2">
         <v>84</v>
@@ -3298,7 +3616,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>